<commit_message>
DBG TO MCU RX_ TX issue fixed
</commit_message>
<xml_diff>
--- a/PCB_project/Jewel_ESP32/Project Outputs for Jewel_ESP32/BOM/Bill of Materials-Jewel_ESP32.xlsx
+++ b/PCB_project/Jewel_ESP32/Project Outputs for Jewel_ESP32/BOM/Bill of Materials-Jewel_ESP32.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahksh\OneDrive\Documents\GitHub\Jewel_Controller\PCB_project\Jewel_ESP32\Project Outputs for Jewel_ESP32\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C62AC0F6-C7B6-4FE4-855F-499D49E26C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B718A2C9-EFA1-4F23-8992-D7C4327880D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{C7EC4349-0A25-4F9A-AAC8-AD6ED7290C25}"/>
+    <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{6DA219F3-7498-4754-85CD-E6979C30EE25}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Jewel_ESP32" sheetId="1" r:id="rId1"/>
@@ -1037,7 +1037,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{862BE3C0-CDCD-401C-BE05-55C29F93D75B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DD9CA4C-D5DD-460E-BA20-750F54116F7B}">
   <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>